<commit_message>
2026 world cup teams finalized
</commit_message>
<xml_diff>
--- a/src/stp/database/2026-mens-world-cup.xlsx
+++ b/src/stp/database/2026-mens-world-cup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bruceoberg/code/soccer-tourney-poster/src/stp/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E053B6F-5B47-BF4F-A60C-4CE17B38AB68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC48D30B-3460-A940-AE99-20D8AC909567}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19280" activeTab="1" xr2:uid="{51C3DE88-701F-4CAC-8963-452186F7FFBA}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19280" activeTab="2" xr2:uid="{51C3DE88-701F-4CAC-8963-452186F7FFBA}"/>
   </bookViews>
   <sheets>
     <sheet name="Properties" sheetId="13" r:id="rId1"/>
@@ -592,30 +592,18 @@
     <t>SAF</t>
   </si>
   <si>
-    <t>??D</t>
-  </si>
-  <si>
-    <t>??A</t>
-  </si>
-  <si>
     <t>HAI</t>
   </si>
   <si>
     <t>PAR</t>
   </si>
   <si>
-    <t>??C</t>
-  </si>
-  <si>
     <t>CUW</t>
   </si>
   <si>
     <t>CIV</t>
   </si>
   <si>
-    <t>??B</t>
-  </si>
-  <si>
     <t>NZL</t>
   </si>
   <si>
@@ -625,15 +613,9 @@
     <t>KSA</t>
   </si>
   <si>
-    <t>??2</t>
-  </si>
-  <si>
     <t>JOR</t>
   </si>
   <si>
-    <t>??1</t>
-  </si>
-  <si>
     <t>GHA</t>
   </si>
   <si>
@@ -797,6 +779,24 @@
   </si>
   <si>
     <t>after-extra-time</t>
+  </si>
+  <si>
+    <t>CZE</t>
+  </si>
+  <si>
+    <t>TUR</t>
+  </si>
+  <si>
+    <t>SWE</t>
+  </si>
+  <si>
+    <t>IRQ</t>
+  </si>
+  <si>
+    <t>BIH</t>
+  </si>
+  <si>
+    <t>COD</t>
   </si>
 </sst>
 </file>
@@ -953,9 +953,9 @@
     <tableColumn id="12" xr3:uid="{AC0139B3-7839-F243-81F2-C8F8601CBDE1}" name="away-team"/>
     <tableColumn id="6" xr3:uid="{A0CDBBB6-1128-45BC-8300-89FE399860C1}" name="home-score" dataDxfId="4"/>
     <tableColumn id="9" xr3:uid="{95DA1082-F87D-4A64-B45A-77AEEA888386}" name="away-score" dataDxfId="3"/>
-    <tableColumn id="14" xr3:uid="{AF9504D2-0653-5049-AD21-E4B2A9F7499E}" name="after-extra-time" dataDxfId="0"/>
-    <tableColumn id="8" xr3:uid="{5865175D-2339-4B50-A707-595597D0BEF5}" name="home-tiebreaker" dataDxfId="2"/>
-    <tableColumn id="7" xr3:uid="{967E27DF-151D-40C4-9623-59691A5D7311}" name="away-tiebreaker" dataDxfId="1"/>
+    <tableColumn id="14" xr3:uid="{AF9504D2-0653-5049-AD21-E4B2A9F7499E}" name="after-extra-time" dataDxfId="2"/>
+    <tableColumn id="8" xr3:uid="{5865175D-2339-4B50-A707-595597D0BEF5}" name="home-tiebreaker" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{967E27DF-151D-40C4-9623-59691A5D7311}" name="away-tiebreaker" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1284,7 +1284,7 @@
         <v>54</v>
       </c>
       <c r="B1" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="C1" t="s">
         <v>65</v>
@@ -1292,18 +1292,18 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>239</v>
+        <v>233</v>
       </c>
       <c r="B2" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>240</v>
+        <v>234</v>
       </c>
       <c r="B3" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -1311,23 +1311,23 @@
         <v>75</v>
       </c>
       <c r="B4" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
       <c r="B5" t="s">
         <v>70</v>
       </c>
       <c r="C5" t="s">
-        <v>236</v>
+        <v>230</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
       <c r="B6" t="s">
         <v>69</v>
@@ -1338,7 +1338,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
       <c r="B7" t="s">
         <v>68</v>
@@ -1349,7 +1349,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
       <c r="B8" t="s">
         <v>71</v>
@@ -1360,7 +1360,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
       <c r="B9" t="s">
         <v>72</v>
@@ -1371,7 +1371,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
       <c r="B10" t="s">
         <v>135</v>
@@ -1382,7 +1382,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
       <c r="B11" t="s">
         <v>129</v>
@@ -1393,18 +1393,18 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="B12" t="s">
         <v>67</v>
       </c>
       <c r="C12" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
       <c r="B13" t="s">
         <v>73</v>
@@ -1415,18 +1415,18 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
       <c r="B14" t="s">
         <v>134</v>
       </c>
       <c r="C14" t="s">
-        <v>237</v>
+        <v>231</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="B15" t="s">
         <v>74</v>
@@ -1437,85 +1437,85 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
       <c r="B16" t="s">
         <v>136</v>
       </c>
       <c r="C16" t="s">
-        <v>238</v>
+        <v>232</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>241</v>
+        <v>235</v>
       </c>
       <c r="B17" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>242</v>
+        <v>236</v>
       </c>
       <c r="B18" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>243</v>
+        <v>237</v>
       </c>
       <c r="B19" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="B20" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>245</v>
+        <v>239</v>
       </c>
       <c r="B21" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>246</v>
+        <v>240</v>
       </c>
       <c r="B22" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>247</v>
+        <v>241</v>
       </c>
       <c r="B23" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>248</v>
+        <v>242</v>
       </c>
       <c r="B24" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="B25" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
@@ -1523,7 +1523,7 @@
         <v>64</v>
       </c>
       <c r="B26" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
@@ -1531,7 +1531,7 @@
         <v>66</v>
       </c>
       <c r="B27" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
@@ -1539,7 +1539,7 @@
         <v>76</v>
       </c>
       <c r="B28" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
@@ -1547,7 +1547,7 @@
         <v>77</v>
       </c>
       <c r="B29" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
@@ -1555,7 +1555,7 @@
         <v>78</v>
       </c>
       <c r="B30" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
@@ -1563,7 +1563,7 @@
         <v>79</v>
       </c>
       <c r="B31" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
@@ -1571,7 +1571,7 @@
         <v>80</v>
       </c>
       <c r="B32" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
     </row>
   </sheetData>
@@ -1613,10 +1613,10 @@
         <v>50</v>
       </c>
       <c r="F1" t="s">
-        <v>250</v>
+        <v>244</v>
       </c>
       <c r="G1" t="s">
-        <v>251</v>
+        <v>245</v>
       </c>
       <c r="H1" t="s">
         <v>62</v>
@@ -1631,7 +1631,7 @@
         <v>56</v>
       </c>
       <c r="L1" t="s">
-        <v>252</v>
+        <v>246</v>
       </c>
       <c r="M1" t="s">
         <v>58</v>
@@ -1687,7 +1687,7 @@
       </c>
       <c r="G3" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[away-seed]],seeds[seed],0)),"")</f>
-        <v>??D</v>
+        <v>CZE</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.2">
@@ -1712,7 +1712,7 @@
       </c>
       <c r="G4" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[away-seed]],seeds[seed],0)),"")</f>
-        <v>??A</v>
+        <v>BIH</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.2">
@@ -1787,7 +1787,7 @@
       </c>
       <c r="G7" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[away-seed]],seeds[seed],0)),"")</f>
-        <v>??C</v>
+        <v>TUR</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.2">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="F13" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[home-seed]],seeds[seed],0)),"")</f>
-        <v>??B</v>
+        <v>SWE</v>
       </c>
       <c r="G13" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[away-seed]],seeds[seed],0)),"")</f>
@@ -2083,7 +2083,7 @@
       </c>
       <c r="F19" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[home-seed]],seeds[seed],0)),"")</f>
-        <v>??2</v>
+        <v>IRQ</v>
       </c>
       <c r="G19" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[away-seed]],seeds[seed],0)),"")</f>
@@ -2212,7 +2212,7 @@
       </c>
       <c r="G24" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[away-seed]],seeds[seed],0)),"")</f>
-        <v>??1</v>
+        <v>COD</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.2">
@@ -2258,7 +2258,7 @@
       </c>
       <c r="F26" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[home-seed]],seeds[seed],0)),"")</f>
-        <v>??D</v>
+        <v>CZE</v>
       </c>
       <c r="G26" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[away-seed]],seeds[seed],0)),"")</f>
@@ -2287,7 +2287,7 @@
       </c>
       <c r="G27" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[away-seed]],seeds[seed],0)),"")</f>
-        <v>??A</v>
+        <v>BIH</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.2">
@@ -2408,7 +2408,7 @@
       </c>
       <c r="F32" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[home-seed]],seeds[seed],0)),"")</f>
-        <v>??C</v>
+        <v>TUR</v>
       </c>
       <c r="G32" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[away-seed]],seeds[seed],0)),"")</f>
@@ -2512,7 +2512,7 @@
       </c>
       <c r="G36" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[away-seed]],seeds[seed],0)),"")</f>
-        <v>??B</v>
+        <v>SWE</v>
       </c>
     </row>
     <row r="37" spans="1:7" x14ac:dyDescent="0.2">
@@ -2687,7 +2687,7 @@
       </c>
       <c r="G43" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[away-seed]],seeds[seed],0)),"")</f>
-        <v>??2</v>
+        <v>IRQ</v>
       </c>
     </row>
     <row r="44" spans="1:7" x14ac:dyDescent="0.2">
@@ -2837,7 +2837,7 @@
       </c>
       <c r="G49" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[away-seed]],seeds[seed],0)),"")</f>
-        <v>??1</v>
+        <v>COD</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.2">
@@ -2933,7 +2933,7 @@
       </c>
       <c r="F53" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[home-seed]],seeds[seed],0)),"")</f>
-        <v>??A</v>
+        <v>BIH</v>
       </c>
       <c r="G53" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[away-seed]],seeds[seed],0)),"")</f>
@@ -2958,7 +2958,7 @@
       </c>
       <c r="F54" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[home-seed]],seeds[seed],0)),"")</f>
-        <v>??D</v>
+        <v>CZE</v>
       </c>
       <c r="G54" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[away-seed]],seeds[seed],0)),"")</f>
@@ -3062,7 +3062,7 @@
       </c>
       <c r="G58" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[away-seed]],seeds[seed],0)),"")</f>
-        <v>??B</v>
+        <v>SWE</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">
@@ -3108,7 +3108,7 @@
       </c>
       <c r="F60" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[home-seed]],seeds[seed],0)),"")</f>
-        <v>??C</v>
+        <v>TUR</v>
       </c>
       <c r="G60" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[away-seed]],seeds[seed],0)),"")</f>
@@ -3187,7 +3187,7 @@
       </c>
       <c r="G63" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[away-seed]],seeds[seed],0)),"")</f>
-        <v>??2</v>
+        <v>IRQ</v>
       </c>
     </row>
     <row r="64" spans="1:7" x14ac:dyDescent="0.2">
@@ -3433,7 +3433,7 @@
       </c>
       <c r="F73" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[home-seed]],seeds[seed],0)),"")</f>
-        <v>??1</v>
+        <v>COD</v>
       </c>
       <c r="G73" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[away-seed]],seeds[seed],0)),"")</f>
@@ -4195,10 +4195,10 @@
         <v>103</v>
       </c>
       <c r="B104" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
       <c r="C104" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="D104" s="4">
         <v>46221.875</v>
@@ -4292,7 +4292,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>184</v>
+        <v>247</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -4308,7 +4308,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>185</v>
+        <v>251</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -4348,7 +4348,7 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
@@ -4372,7 +4372,7 @@
         <v>9</v>
       </c>
       <c r="B15" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
@@ -4388,7 +4388,7 @@
         <v>11</v>
       </c>
       <c r="B17" t="s">
-        <v>188</v>
+        <v>248</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
@@ -4404,7 +4404,7 @@
         <v>19</v>
       </c>
       <c r="B19" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
@@ -4412,7 +4412,7 @@
         <v>20</v>
       </c>
       <c r="B20" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
@@ -4444,7 +4444,7 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>191</v>
+        <v>249</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
@@ -4484,7 +4484,7 @@
         <v>25</v>
       </c>
       <c r="B29" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
@@ -4500,7 +4500,7 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
@@ -4508,7 +4508,7 @@
         <v>26</v>
       </c>
       <c r="B32" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
@@ -4540,7 +4540,7 @@
         <v>105</v>
       </c>
       <c r="B36" t="s">
-        <v>195</v>
+        <v>250</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
@@ -4580,7 +4580,7 @@
         <v>110</v>
       </c>
       <c r="B41" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
@@ -4596,7 +4596,7 @@
         <v>112</v>
       </c>
       <c r="B43" t="s">
-        <v>197</v>
+        <v>252</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
@@ -4604,7 +4604,7 @@
         <v>113</v>
       </c>
       <c r="B44" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
@@ -4636,7 +4636,7 @@
         <v>117</v>
       </c>
       <c r="B48" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
@@ -4644,7 +4644,7 @@
         <v>118</v>
       </c>
       <c r="B49" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
inverse group sets shown with parens, not tildes
- also some group hinting expeimentation.
</commit_message>
<xml_diff>
--- a/src/stp/database/2026-mens-world-cup.xlsx
+++ b/src/stp/database/2026-mens-world-cup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bruceoberg/code/soccer-tourney-poster/src/stp/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC48D30B-3460-A940-AE99-20D8AC909567}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5ADDDE84-D666-6348-AE7E-F73E6647AC5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19280" activeTab="2" xr2:uid="{51C3DE88-701F-4CAC-8963-452186F7FFBA}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19280" activeTab="1" xr2:uid="{51C3DE88-701F-4CAC-8963-452186F7FFBA}"/>
   </bookViews>
   <sheets>
     <sheet name="Properties" sheetId="13" r:id="rId1"/>
@@ -589,9 +589,6 @@
     <t>W102</t>
   </si>
   <si>
-    <t>SAF</t>
-  </si>
-  <si>
     <t>HAI</t>
   </si>
   <si>
@@ -797,6 +794,9 @@
   </si>
   <si>
     <t>COD</t>
+  </si>
+  <si>
+    <t>RSA</t>
   </si>
 </sst>
 </file>
@@ -1284,7 +1284,7 @@
         <v>54</v>
       </c>
       <c r="B1" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C1" t="s">
         <v>65</v>
@@ -1292,18 +1292,18 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B2" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B3" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -1311,23 +1311,23 @@
         <v>75</v>
       </c>
       <c r="B4" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B5" t="s">
         <v>70</v>
       </c>
       <c r="C5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B6" t="s">
         <v>69</v>
@@ -1338,7 +1338,7 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B7" t="s">
         <v>68</v>
@@ -1349,7 +1349,7 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B8" t="s">
         <v>71</v>
@@ -1360,7 +1360,7 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B9" t="s">
         <v>72</v>
@@ -1371,7 +1371,7 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B10" t="s">
         <v>135</v>
@@ -1382,7 +1382,7 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B11" t="s">
         <v>129</v>
@@ -1393,18 +1393,18 @@
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B12" t="s">
         <v>67</v>
       </c>
       <c r="C12" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B13" t="s">
         <v>73</v>
@@ -1415,18 +1415,18 @@
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B14" t="s">
         <v>134</v>
       </c>
       <c r="C14" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B15" t="s">
         <v>74</v>
@@ -1437,85 +1437,85 @@
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B16" t="s">
         <v>136</v>
       </c>
       <c r="C16" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B17" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B18" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B19" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B20" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B21" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B22" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B23" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B24" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B25" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
@@ -1523,7 +1523,7 @@
         <v>64</v>
       </c>
       <c r="B26" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
@@ -1531,7 +1531,7 @@
         <v>66</v>
       </c>
       <c r="B27" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
@@ -1539,7 +1539,7 @@
         <v>76</v>
       </c>
       <c r="B28" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
@@ -1547,7 +1547,7 @@
         <v>77</v>
       </c>
       <c r="B29" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
@@ -1555,7 +1555,7 @@
         <v>78</v>
       </c>
       <c r="B30" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
@@ -1563,7 +1563,7 @@
         <v>79</v>
       </c>
       <c r="B31" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
@@ -1571,7 +1571,7 @@
         <v>80</v>
       </c>
       <c r="B32" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
   </sheetData>
@@ -1613,10 +1613,10 @@
         <v>50</v>
       </c>
       <c r="F1" t="s">
+        <v>243</v>
+      </c>
+      <c r="G1" t="s">
         <v>244</v>
-      </c>
-      <c r="G1" t="s">
-        <v>245</v>
       </c>
       <c r="H1" t="s">
         <v>62</v>
@@ -1631,7 +1631,7 @@
         <v>56</v>
       </c>
       <c r="L1" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="M1" t="s">
         <v>58</v>
@@ -1662,7 +1662,7 @@
       </c>
       <c r="G2" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[away-seed]],seeds[seed],0)),"")</f>
-        <v>SAF</v>
+        <v>RSA</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.2">
@@ -1776,7 +1776,7 @@
         <v>11</v>
       </c>
       <c r="D7" s="4">
-        <v>46186.166666666664</v>
+        <v>46187.166666666664</v>
       </c>
       <c r="E7">
         <v>1</v>
@@ -2126,7 +2126,7 @@
         <v>110</v>
       </c>
       <c r="D21" s="4">
-        <v>46189.166666666664</v>
+        <v>46190.166666666664</v>
       </c>
       <c r="E21">
         <v>11</v>
@@ -2262,7 +2262,7 @@
       </c>
       <c r="G26" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[away-seed]],seeds[seed],0)),"")</f>
-        <v>SAF</v>
+        <v>RSA</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.2">
@@ -2351,7 +2351,7 @@
         <v>12</v>
       </c>
       <c r="D30" s="4">
-        <v>46193.041666666664</v>
+        <v>46193.020833333336</v>
       </c>
       <c r="E30">
         <v>9</v>
@@ -2401,7 +2401,7 @@
         <v>9</v>
       </c>
       <c r="D32" s="4">
-        <v>46192.166666666664</v>
+        <v>46193.125</v>
       </c>
       <c r="E32">
         <v>11</v>
@@ -2526,7 +2526,7 @@
         <v>17</v>
       </c>
       <c r="D37" s="4">
-        <v>46193.166666666664</v>
+        <v>46194.166666666664</v>
       </c>
       <c r="E37">
         <v>16</v>
@@ -2983,7 +2983,7 @@
       </c>
       <c r="F55" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[home-seed]],seeds[seed],0)),"")</f>
-        <v>SAF</v>
+        <v>RSA</v>
       </c>
       <c r="G55" t="str">
         <f>_xlfn.IFNA(INDEX(seeds[team],MATCH(matches[[#This Row],[away-seed]],seeds[seed],0)),"")</f>
@@ -4195,10 +4195,10 @@
         <v>103</v>
       </c>
       <c r="B104" t="s">
+        <v>194</v>
+      </c>
+      <c r="C104" t="s">
         <v>195</v>
-      </c>
-      <c r="C104" t="s">
-        <v>196</v>
       </c>
       <c r="D104" s="4">
         <v>46221.875</v>
@@ -4276,7 +4276,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>183</v>
+        <v>252</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -4292,7 +4292,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -4308,7 +4308,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -4348,7 +4348,7 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
@@ -4372,7 +4372,7 @@
         <v>9</v>
       </c>
       <c r="B15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
@@ -4388,7 +4388,7 @@
         <v>11</v>
       </c>
       <c r="B17" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
@@ -4404,7 +4404,7 @@
         <v>19</v>
       </c>
       <c r="B19" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
@@ -4412,7 +4412,7 @@
         <v>20</v>
       </c>
       <c r="B20" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
@@ -4444,7 +4444,7 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
@@ -4484,7 +4484,7 @@
         <v>25</v>
       </c>
       <c r="B29" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
@@ -4500,7 +4500,7 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
@@ -4508,7 +4508,7 @@
         <v>26</v>
       </c>
       <c r="B32" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
@@ -4540,7 +4540,7 @@
         <v>105</v>
       </c>
       <c r="B36" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
@@ -4580,7 +4580,7 @@
         <v>110</v>
       </c>
       <c r="B41" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
@@ -4596,7 +4596,7 @@
         <v>112</v>
       </c>
       <c r="B43" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
@@ -4604,7 +4604,7 @@
         <v>113</v>
       </c>
       <c r="B44" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
@@ -4636,7 +4636,7 @@
         <v>117</v>
       </c>
       <c r="B48" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
@@ -4644,7 +4644,7 @@
         <v>118</v>
       </c>
       <c r="B49" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
remove dashes from 3rd place elimination slot labels (to match official listings)
</commit_message>
<xml_diff>
--- a/src/stp/database/2026-mens-world-cup.xlsx
+++ b/src/stp/database/2026-mens-world-cup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bruceoberg/code/soccer-tourney-poster/src/stp/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F918A0D8-8F41-6642-9876-93C3FDDBF9F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D440017-82CA-FE48-8D99-CCD8D6AF4F4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="19280" xr2:uid="{51C3DE88-701F-4CAC-8963-452186F7FFBA}"/>
+    <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="19280" activeTab="1" xr2:uid="{51C3DE88-701F-4CAC-8963-452186F7FFBA}"/>
   </bookViews>
   <sheets>
     <sheet name="Properties" sheetId="13" r:id="rId1"/>
@@ -406,33 +406,15 @@
     <t>teal</t>
   </si>
   <si>
-    <t>3-ABCDF</t>
-  </si>
-  <si>
     <t>1I</t>
   </si>
   <si>
-    <t>3-CDFGH</t>
-  </si>
-  <si>
     <t>2I</t>
   </si>
   <si>
-    <t>3-CEFHI</t>
-  </si>
-  <si>
     <t>1L</t>
   </si>
   <si>
-    <t>3-EHIJK</t>
-  </si>
-  <si>
-    <t>3-BEFIJ</t>
-  </si>
-  <si>
-    <t>3-AEHIJ</t>
-  </si>
-  <si>
     <t>2K</t>
   </si>
   <si>
@@ -442,18 +424,12 @@
     <t>2J</t>
   </si>
   <si>
-    <t>3-EFGIJ</t>
-  </si>
-  <si>
     <t>1J</t>
   </si>
   <si>
     <t>1K</t>
   </si>
   <si>
-    <t>3-DEIJL</t>
-  </si>
-  <si>
     <t>W74</t>
   </si>
   <si>
@@ -797,6 +773,30 @@
   </si>
   <si>
     <t>#e1aab6</t>
+  </si>
+  <si>
+    <t>3ABCDF</t>
+  </si>
+  <si>
+    <t>3CDFGH</t>
+  </si>
+  <si>
+    <t>3CEFHI</t>
+  </si>
+  <si>
+    <t>3EHIJK</t>
+  </si>
+  <si>
+    <t>3BEFIJ</t>
+  </si>
+  <si>
+    <t>3AEHIJ</t>
+  </si>
+  <si>
+    <t>3EFGIJ</t>
+  </si>
+  <si>
+    <t>3DEIJL</t>
   </si>
 </sst>
 </file>
@@ -1284,7 +1284,7 @@
         <v>54</v>
       </c>
       <c r="B1" t="s">
-        <v>200</v>
+        <v>192</v>
       </c>
       <c r="C1" t="s">
         <v>65</v>
@@ -1292,18 +1292,18 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>214</v>
+        <v>206</v>
       </c>
       <c r="B2" t="s">
-        <v>182</v>
+        <v>174</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>215</v>
+        <v>207</v>
       </c>
       <c r="B3" t="s">
-        <v>183</v>
+        <v>175</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.2">
@@ -1311,26 +1311,26 @@
         <v>67</v>
       </c>
       <c r="B4" t="s">
-        <v>181</v>
+        <v>173</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
-        <v>204</v>
+        <v>196</v>
       </c>
       <c r="B5" t="s">
-        <v>241</v>
+        <v>233</v>
       </c>
       <c r="C5" t="s">
-        <v>213</v>
+        <v>205</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
-        <v>203</v>
+        <v>195</v>
       </c>
       <c r="B6" t="s">
-        <v>249</v>
+        <v>241</v>
       </c>
       <c r="C6" t="s">
         <v>118</v>
@@ -1338,10 +1338,10 @@
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
-        <v>202</v>
+        <v>194</v>
       </c>
       <c r="B7" t="s">
-        <v>242</v>
+        <v>234</v>
       </c>
       <c r="C7" t="s">
         <v>117</v>
@@ -1349,10 +1349,10 @@
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
-        <v>205</v>
+        <v>197</v>
       </c>
       <c r="B8" t="s">
-        <v>243</v>
+        <v>235</v>
       </c>
       <c r="C8" t="s">
         <v>119</v>
@@ -1360,10 +1360,10 @@
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
-        <v>207</v>
+        <v>199</v>
       </c>
       <c r="B9" t="s">
-        <v>244</v>
+        <v>236</v>
       </c>
       <c r="C9" t="s">
         <v>120</v>
@@ -1371,10 +1371,10 @@
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
-        <v>210</v>
+        <v>202</v>
       </c>
       <c r="B10" t="s">
-        <v>245</v>
+        <v>237</v>
       </c>
       <c r="C10" t="s">
         <v>121</v>
@@ -1382,140 +1382,140 @@
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
-        <v>211</v>
+        <v>203</v>
       </c>
       <c r="B11" t="s">
-        <v>246</v>
+        <v>238</v>
       </c>
       <c r="C11" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
-        <v>201</v>
+        <v>193</v>
       </c>
       <c r="B12" t="s">
-        <v>247</v>
+        <v>239</v>
       </c>
       <c r="C12" t="s">
-        <v>236</v>
+        <v>228</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
-        <v>208</v>
+        <v>200</v>
       </c>
       <c r="B13" t="s">
-        <v>248</v>
+        <v>240</v>
       </c>
       <c r="C13" t="s">
-        <v>237</v>
+        <v>229</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
-        <v>209</v>
+        <v>201</v>
       </c>
       <c r="B14" t="s">
-        <v>250</v>
+        <v>242</v>
       </c>
       <c r="C14" t="s">
-        <v>238</v>
+        <v>230</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>206</v>
+        <v>198</v>
       </c>
       <c r="B15" t="s">
-        <v>251</v>
+        <v>243</v>
       </c>
       <c r="C15" t="s">
-        <v>239</v>
+        <v>231</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
-        <v>212</v>
+        <v>204</v>
       </c>
       <c r="B16" t="s">
-        <v>252</v>
+        <v>244</v>
       </c>
       <c r="C16" t="s">
-        <v>240</v>
+        <v>232</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
-        <v>216</v>
+        <v>208</v>
       </c>
       <c r="B17" t="s">
-        <v>184</v>
+        <v>176</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
-        <v>217</v>
+        <v>209</v>
       </c>
       <c r="B18" t="s">
-        <v>185</v>
+        <v>177</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>218</v>
+        <v>210</v>
       </c>
       <c r="B19" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>219</v>
+        <v>211</v>
       </c>
       <c r="B20" t="s">
-        <v>187</v>
+        <v>179</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>220</v>
+        <v>212</v>
       </c>
       <c r="B21" t="s">
-        <v>188</v>
+        <v>180</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>221</v>
+        <v>213</v>
       </c>
       <c r="B22" t="s">
-        <v>189</v>
+        <v>181</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>222</v>
+        <v>214</v>
       </c>
       <c r="B23" t="s">
-        <v>190</v>
+        <v>182</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>223</v>
+        <v>215</v>
       </c>
       <c r="B24" t="s">
-        <v>191</v>
+        <v>183</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="B25" t="s">
-        <v>192</v>
+        <v>184</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.2">
@@ -1523,7 +1523,7 @@
         <v>64</v>
       </c>
       <c r="B26" t="s">
-        <v>193</v>
+        <v>185</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.2">
@@ -1531,7 +1531,7 @@
         <v>66</v>
       </c>
       <c r="B27" t="s">
-        <v>194</v>
+        <v>186</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.2">
@@ -1539,7 +1539,7 @@
         <v>68</v>
       </c>
       <c r="B28" t="s">
-        <v>195</v>
+        <v>187</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.2">
@@ -1547,7 +1547,7 @@
         <v>69</v>
       </c>
       <c r="B29" t="s">
-        <v>196</v>
+        <v>188</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
@@ -1555,7 +1555,7 @@
         <v>70</v>
       </c>
       <c r="B30" t="s">
-        <v>197</v>
+        <v>189</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.2">
@@ -1563,7 +1563,7 @@
         <v>71</v>
       </c>
       <c r="B31" t="s">
-        <v>198</v>
+        <v>190</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
@@ -1571,7 +1571,7 @@
         <v>72</v>
       </c>
       <c r="B32" t="s">
-        <v>199</v>
+        <v>191</v>
       </c>
     </row>
   </sheetData>
@@ -1614,10 +1614,10 @@
         <v>50</v>
       </c>
       <c r="F1" t="s">
-        <v>225</v>
+        <v>217</v>
       </c>
       <c r="G1" t="s">
-        <v>226</v>
+        <v>218</v>
       </c>
       <c r="H1" t="s">
         <v>62</v>
@@ -1632,7 +1632,7 @@
         <v>56</v>
       </c>
       <c r="L1" t="s">
-        <v>227</v>
+        <v>219</v>
       </c>
       <c r="M1" t="s">
         <v>58</v>
@@ -3474,7 +3474,7 @@
         <v>40</v>
       </c>
       <c r="C75" t="s">
-        <v>122</v>
+        <v>245</v>
       </c>
       <c r="D75" s="4">
         <v>46202.854166666664</v>
@@ -3546,10 +3546,10 @@
         <v>77</v>
       </c>
       <c r="B78" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C78" t="s">
-        <v>124</v>
+        <v>246</v>
       </c>
       <c r="D78" s="4">
         <v>46203.875</v>
@@ -3574,7 +3574,7 @@
         <v>45</v>
       </c>
       <c r="C79" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="D79" s="4">
         <v>46203.708333333328</v>
@@ -3599,7 +3599,7 @@
         <v>32</v>
       </c>
       <c r="C80" t="s">
-        <v>126</v>
+        <v>247</v>
       </c>
       <c r="D80" s="4">
         <v>46204.041666666664</v>
@@ -3621,10 +3621,10 @@
         <v>80</v>
       </c>
       <c r="B81" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C81" t="s">
-        <v>128</v>
+        <v>248</v>
       </c>
       <c r="D81" s="4">
         <v>46204.666666666664</v>
@@ -3649,7 +3649,7 @@
         <v>38</v>
       </c>
       <c r="C82" t="s">
-        <v>129</v>
+        <v>249</v>
       </c>
       <c r="D82" s="4">
         <v>46205</v>
@@ -3674,7 +3674,7 @@
         <v>42</v>
       </c>
       <c r="C83" t="s">
-        <v>130</v>
+        <v>250</v>
       </c>
       <c r="D83" s="4">
         <v>46204.833333333328</v>
@@ -3696,10 +3696,10 @@
         <v>83</v>
       </c>
       <c r="B84" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="C84" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="D84" s="4">
         <v>46205.958333333328</v>
@@ -3724,7 +3724,7 @@
         <v>46</v>
       </c>
       <c r="C85" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="D85" s="4">
         <v>46205.791666666664</v>
@@ -3749,7 +3749,7 @@
         <v>36</v>
       </c>
       <c r="C86" t="s">
-        <v>134</v>
+        <v>251</v>
       </c>
       <c r="D86" s="4">
         <v>46206.125</v>
@@ -3771,7 +3771,7 @@
         <v>86</v>
       </c>
       <c r="B87" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="C87" t="s">
         <v>43</v>
@@ -3796,10 +3796,10 @@
         <v>87</v>
       </c>
       <c r="B88" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="C88" t="s">
-        <v>137</v>
+        <v>252</v>
       </c>
       <c r="D88" s="4">
         <v>46207.0625</v>
@@ -3846,10 +3846,10 @@
         <v>89</v>
       </c>
       <c r="B90" t="s">
-        <v>138</v>
+        <v>130</v>
       </c>
       <c r="C90" t="s">
-        <v>139</v>
+        <v>131</v>
       </c>
       <c r="D90" s="4">
         <v>46207.875</v>
@@ -3871,10 +3871,10 @@
         <v>90</v>
       </c>
       <c r="B91" t="s">
-        <v>140</v>
+        <v>132</v>
       </c>
       <c r="C91" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="D91" s="4">
         <v>46207.708333333328</v>
@@ -3896,10 +3896,10 @@
         <v>91</v>
       </c>
       <c r="B92" t="s">
-        <v>142</v>
+        <v>134</v>
       </c>
       <c r="C92" t="s">
-        <v>143</v>
+        <v>135</v>
       </c>
       <c r="D92" s="4">
         <v>46208.833333333328</v>
@@ -3921,10 +3921,10 @@
         <v>92</v>
       </c>
       <c r="B93" t="s">
-        <v>144</v>
+        <v>136</v>
       </c>
       <c r="C93" t="s">
-        <v>145</v>
+        <v>137</v>
       </c>
       <c r="D93" s="4">
         <v>46209</v>
@@ -3946,10 +3946,10 @@
         <v>93</v>
       </c>
       <c r="B94" t="s">
-        <v>146</v>
+        <v>138</v>
       </c>
       <c r="C94" t="s">
-        <v>147</v>
+        <v>139</v>
       </c>
       <c r="D94" s="4">
         <v>46209.791666666664</v>
@@ -3971,10 +3971,10 @@
         <v>94</v>
       </c>
       <c r="B95" t="s">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="C95" t="s">
-        <v>149</v>
+        <v>141</v>
       </c>
       <c r="D95" s="4">
         <v>46210</v>
@@ -3996,10 +3996,10 @@
         <v>95</v>
       </c>
       <c r="B96" t="s">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="C96" t="s">
-        <v>151</v>
+        <v>143</v>
       </c>
       <c r="D96" s="4">
         <v>46210.666666666664</v>
@@ -4021,10 +4021,10 @@
         <v>96</v>
       </c>
       <c r="B97" t="s">
-        <v>152</v>
+        <v>144</v>
       </c>
       <c r="C97" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="D97" s="4">
         <v>46210.833333333328</v>
@@ -4046,10 +4046,10 @@
         <v>97</v>
       </c>
       <c r="B98" t="s">
-        <v>154</v>
+        <v>146</v>
       </c>
       <c r="C98" t="s">
-        <v>155</v>
+        <v>147</v>
       </c>
       <c r="D98" s="4">
         <v>46212.833333333328</v>
@@ -4071,10 +4071,10 @@
         <v>98</v>
       </c>
       <c r="B99" t="s">
-        <v>156</v>
+        <v>148</v>
       </c>
       <c r="C99" t="s">
-        <v>157</v>
+        <v>149</v>
       </c>
       <c r="D99" s="4">
         <v>46213.791666666664</v>
@@ -4096,10 +4096,10 @@
         <v>99</v>
       </c>
       <c r="B100" t="s">
-        <v>158</v>
+        <v>150</v>
       </c>
       <c r="C100" t="s">
-        <v>159</v>
+        <v>151</v>
       </c>
       <c r="D100" s="4">
         <v>46214.875</v>
@@ -4121,10 +4121,10 @@
         <v>100</v>
       </c>
       <c r="B101" t="s">
-        <v>160</v>
+        <v>152</v>
       </c>
       <c r="C101" t="s">
-        <v>161</v>
+        <v>153</v>
       </c>
       <c r="D101" s="4">
         <v>46215.041666666664</v>
@@ -4146,10 +4146,10 @@
         <v>101</v>
       </c>
       <c r="B102" t="s">
-        <v>162</v>
+        <v>154</v>
       </c>
       <c r="C102" t="s">
-        <v>163</v>
+        <v>155</v>
       </c>
       <c r="D102" s="4">
         <v>46217.791666666664</v>
@@ -4171,10 +4171,10 @@
         <v>102</v>
       </c>
       <c r="B103" t="s">
-        <v>164</v>
+        <v>156</v>
       </c>
       <c r="C103" t="s">
-        <v>165</v>
+        <v>157</v>
       </c>
       <c r="D103" s="4">
         <v>46218.791666666664</v>
@@ -4196,10 +4196,10 @@
         <v>103</v>
       </c>
       <c r="B104" t="s">
-        <v>179</v>
+        <v>171</v>
       </c>
       <c r="C104" t="s">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="D104" s="4">
         <v>46221.875</v>
@@ -4221,10 +4221,10 @@
         <v>104</v>
       </c>
       <c r="B105" t="s">
-        <v>166</v>
+        <v>158</v>
       </c>
       <c r="C105" t="s">
-        <v>167</v>
+        <v>159</v>
       </c>
       <c r="D105" s="4">
         <v>46222.791666666664</v>
@@ -4277,7 +4277,7 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.2">
@@ -4293,7 +4293,7 @@
         <v>3</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>228</v>
+        <v>220</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.2">
@@ -4309,7 +4309,7 @@
         <v>5</v>
       </c>
       <c r="B7" t="s">
-        <v>232</v>
+        <v>224</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.2">
@@ -4349,7 +4349,7 @@
         <v>12</v>
       </c>
       <c r="B12" t="s">
-        <v>168</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.2">
@@ -4373,7 +4373,7 @@
         <v>9</v>
       </c>
       <c r="B15" t="s">
-        <v>169</v>
+        <v>161</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.2">
@@ -4389,7 +4389,7 @@
         <v>11</v>
       </c>
       <c r="B17" t="s">
-        <v>229</v>
+        <v>221</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.2">
@@ -4405,7 +4405,7 @@
         <v>19</v>
       </c>
       <c r="B19" t="s">
-        <v>170</v>
+        <v>162</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.2">
@@ -4413,7 +4413,7 @@
         <v>20</v>
       </c>
       <c r="B20" t="s">
-        <v>171</v>
+        <v>163</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.2">
@@ -4445,7 +4445,7 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.2">
@@ -4485,7 +4485,7 @@
         <v>25</v>
       </c>
       <c r="B29" t="s">
-        <v>172</v>
+        <v>164</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.2">
@@ -4501,7 +4501,7 @@
         <v>29</v>
       </c>
       <c r="B31" t="s">
-        <v>173</v>
+        <v>165</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.2">
@@ -4509,7 +4509,7 @@
         <v>26</v>
       </c>
       <c r="B32" t="s">
-        <v>174</v>
+        <v>166</v>
       </c>
     </row>
     <row r="33" spans="1:2" x14ac:dyDescent="0.2">
@@ -4541,7 +4541,7 @@
         <v>97</v>
       </c>
       <c r="B36" t="s">
-        <v>231</v>
+        <v>223</v>
       </c>
     </row>
     <row r="37" spans="1:2" x14ac:dyDescent="0.2">
@@ -4581,7 +4581,7 @@
         <v>102</v>
       </c>
       <c r="B41" t="s">
-        <v>175</v>
+        <v>167</v>
       </c>
     </row>
     <row r="42" spans="1:2" x14ac:dyDescent="0.2">
@@ -4597,7 +4597,7 @@
         <v>104</v>
       </c>
       <c r="B43" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
     </row>
     <row r="44" spans="1:2" x14ac:dyDescent="0.2">
@@ -4605,7 +4605,7 @@
         <v>105</v>
       </c>
       <c r="B44" t="s">
-        <v>178</v>
+        <v>170</v>
       </c>
     </row>
     <row r="45" spans="1:2" x14ac:dyDescent="0.2">
@@ -4637,7 +4637,7 @@
         <v>109</v>
       </c>
       <c r="B48" t="s">
-        <v>176</v>
+        <v>168</v>
       </c>
     </row>
     <row r="49" spans="1:2" x14ac:dyDescent="0.2">
@@ -4645,7 +4645,7 @@
         <v>110</v>
       </c>
       <c r="B49" t="s">
-        <v>177</v>
+        <v>169</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
corrected blue and purple group colors
</commit_message>
<xml_diff>
--- a/src/stp/database/2026-mens-world-cup.xlsx
+++ b/src/stp/database/2026-mens-world-cup.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bruceoberg/code/soccer-tourney-poster/src/stp/database/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D440017-82CA-FE48-8D99-CCD8D6AF4F4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{768EEF1E-CA39-9B41-9DF5-A37E58750E4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="19280" activeTab="1" xr2:uid="{51C3DE88-701F-4CAC-8963-452186F7FFBA}"/>
+    <workbookView xWindow="0" yWindow="700" windowWidth="34200" windowHeight="19280" xr2:uid="{51C3DE88-701F-4CAC-8963-452186F7FFBA}"/>
   </bookViews>
   <sheets>
     <sheet name="Properties" sheetId="13" r:id="rId1"/>
@@ -745,9 +745,6 @@
     <t>#e9e8b5</t>
   </si>
   <si>
-    <t>#cdd9ff</t>
-  </si>
-  <si>
     <t>#ffc79e</t>
   </si>
   <si>
@@ -760,9 +757,6 @@
     <t>#b5dbe4</t>
   </si>
   <si>
-    <t>#e0d3ff</t>
-  </si>
-  <si>
     <t>#ffbcb9</t>
   </si>
   <si>
@@ -797,6 +791,12 @@
   </si>
   <si>
     <t>3DEIJL</t>
+  </si>
+  <si>
+    <t>#b0d0ee</t>
+  </si>
+  <si>
+    <t>#bbb1d6</t>
   </si>
 </sst>
 </file>
@@ -1330,7 +1330,7 @@
         <v>195</v>
       </c>
       <c r="B6" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="C6" t="s">
         <v>118</v>
@@ -1352,7 +1352,7 @@
         <v>197</v>
       </c>
       <c r="B8" t="s">
-        <v>235</v>
+        <v>251</v>
       </c>
       <c r="C8" t="s">
         <v>119</v>
@@ -1363,7 +1363,7 @@
         <v>199</v>
       </c>
       <c r="B9" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C9" t="s">
         <v>120</v>
@@ -1374,7 +1374,7 @@
         <v>202</v>
       </c>
       <c r="B10" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C10" t="s">
         <v>121</v>
@@ -1385,7 +1385,7 @@
         <v>203</v>
       </c>
       <c r="B11" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="C11" t="s">
         <v>227</v>
@@ -1396,7 +1396,7 @@
         <v>193</v>
       </c>
       <c r="B12" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C12" t="s">
         <v>228</v>
@@ -1407,7 +1407,7 @@
         <v>200</v>
       </c>
       <c r="B13" t="s">
-        <v>240</v>
+        <v>252</v>
       </c>
       <c r="C13" t="s">
         <v>229</v>
@@ -1418,7 +1418,7 @@
         <v>201</v>
       </c>
       <c r="B14" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="C14" t="s">
         <v>230</v>
@@ -1429,7 +1429,7 @@
         <v>198</v>
       </c>
       <c r="B15" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C15" t="s">
         <v>231</v>
@@ -1440,7 +1440,7 @@
         <v>204</v>
       </c>
       <c r="B16" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="C16" t="s">
         <v>232</v>
@@ -3474,7 +3474,7 @@
         <v>40</v>
       </c>
       <c r="C75" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="D75" s="4">
         <v>46202.854166666664</v>
@@ -3549,7 +3549,7 @@
         <v>122</v>
       </c>
       <c r="C78" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="D78" s="4">
         <v>46203.875</v>
@@ -3599,7 +3599,7 @@
         <v>32</v>
       </c>
       <c r="C80" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="D80" s="4">
         <v>46204.041666666664</v>
@@ -3624,7 +3624,7 @@
         <v>124</v>
       </c>
       <c r="C81" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
       <c r="D81" s="4">
         <v>46204.666666666664</v>
@@ -3649,7 +3649,7 @@
         <v>38</v>
       </c>
       <c r="C82" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="D82" s="4">
         <v>46205</v>
@@ -3674,7 +3674,7 @@
         <v>42</v>
       </c>
       <c r="C83" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="D83" s="4">
         <v>46204.833333333328</v>
@@ -3749,7 +3749,7 @@
         <v>36</v>
       </c>
       <c r="C86" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="D86" s="4">
         <v>46206.125</v>
@@ -3799,7 +3799,7 @@
         <v>129</v>
       </c>
       <c r="C88" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="D88" s="4">
         <v>46207.0625</v>

</xml_diff>